<commit_message>
Ground the content proposals and separate issue from change
Drop rewrites whose only difference from the published text was verb
tense or punctuation. MUS 111, 112, and 211 keep their published
descriptions.

New descriptions where the published text does not describe the
course:
- MUS 115, 116, and 215 publish one shared description across three
  levels, as do MUS 118, 119, and 218; each now has a description
  drawn from its own benchmarks in the theory and musicianship guide
- MUS 410 publishes a single sentence naming no content; the proposal
  covers post-tonal collections, pitch-class sets, centricity,
  serialism, form, and the movements after 1945

Formatting: each finding puts the issue on its own line in plain text
with the change beneath it in red, and findings within a cell are
separated by a blank line.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -655,7 +655,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -759,7 +760,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -1192,7 +1194,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -1287,7 +1290,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -1381,50 +1385,7 @@
         <v>2</v>
       </c>
       <c r="T10" s="3" t="inlineStr"/>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>The first of three intensive courses that introduce students to the inner workings of European art music of the 18th and 19th centuries. This course covers diatonic harmony, as well as part-writing, voice-leading, and harmonization techniques.</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Read, write, and analyze the fundamental materials of tonal music using correct terminology and nomenclature. 2. Construct and identify all triad and seventh chord types in root position and inversion. 3. Write four-part (SATB) harmonic progressions using I, V, V⁷, and their inversions, applying basic voice-leading principles. 4. Compose and analyze two-voice counterpoint through fourth species. 5. Apply theoretical concepts at the keyboard and in performance on the student's primary instrument or voice.</t>
-          </r>
-        </is>
-      </c>
+      <c r="U10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1504,50 +1465,7 @@
         <v>2</v>
       </c>
       <c r="T11" s="3" t="inlineStr"/>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>The second of three intensive courses that introduce students to the inner workings of European art music of the 18th and 19th centuries. This course completes diatonic harmony and introduces advanced part-writing, voice-leading, and harmonization techniques.</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Write and analyze SATB progressions using the full vocabulary of diatonic harmony, including all diatonic triads and seventh chords. 2. Identify and apply embellishing chords, the cadential 6/4, and other 6/4 chord types in functional context. 3. Recognize and compose diatonic sequences. 4. Analyze tonal works using Roman numerals, figured bass, and functional labels. 5. Apply diatonic harmonic vocabulary at the keyboard and in performance on the student's primary instrument or voice.</t>
-          </r>
-        </is>
-      </c>
+      <c r="U11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1629,7 +1547,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 118A, renumbered or discontinued → </t>
+            <t xml:space="preserve">requires MUS 118A, renumbered or discontinued
+</t>
           </r>
           <r>
             <rPr>
@@ -1645,15 +1564,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-05-05, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-05-05, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -1673,16 +1586,35 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Sight-sing diatonic melodies in major keys and simple meters using solfège or scale degrees, with accurate pitch, rhythm, and conducting. 2. Take melodic and rhythmic dictation in simple meters, notating pitch and rhythm accurately, including ties and the dotted beat. 3. Detect and correct errors in performed and notated examples. 4. Read fluently across all fifteen major keys.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>First of three concurrent aural skills courses. Sight-singing and dictation of diatonic melodies in major keys and simple meters, rhythmic and pitch notation, error detection, and fluency across all fifteen major keys.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to the other courses in its track, so the levels are indistinguishable in the catalog
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>see the proposed description above</t>
           </r>
         </is>
       </c>
@@ -1771,7 +1703,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 118B, renumbered or discontinued → </t>
+            <t xml:space="preserve">requires MUS 118B, renumbered or discontinued
+</t>
           </r>
           <r>
             <rPr>
@@ -1787,15 +1720,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-05-05, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-05-05, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -1815,16 +1742,35 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Sight-sing diatonic melodies in minor mode, approached through both relative and parallel major and including chromatic 6 and 7 by modal borrowing, and in compound meters, using solfège or scale degrees. 2. Take melodic and rhythmic dictation extending to triplets and duplets, quadruple division in simple meter, sextuple division in compound meter, and syncopation. 3. Perform lower chromatic neighbors and melodic skips to chord tones as prefix neighbors through the tonic, dominant, and subdominant triads. 4. Sing the dominant seventh chord in melodic context.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Second of three concurrent aural skills courses. Sight-singing and dictation in minor mode through relative and parallel major, compound meters, chromatic neighbors and skips to chord tones, triplets and syncopation, and the dominant seventh in melodic context.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to the other courses in its track, so the levels are indistinguishable in the catalog
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>see the proposed description above</t>
           </r>
         </is>
       </c>
@@ -1911,16 +1857,35 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Perform major and minor five-finger patterns and their triads in all common keys. 2. Perform all four triad qualities (major, minor, augmented, diminished) in root position. 3. Play major scales in tetrachord position with correct fingering, and use the damper pedal. 4. Harmonize simple melodies using basic diatonic chords. 5. Sight-read short examples in grand staff at a basic level.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>First of three concurrent keyboard courses for music majors. Major and minor five-finger patterns and their triads, all four triad qualities, major scales in tetrachord position, damper pedal, and basic sight-reading and harmonization.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to the other courses in its track, so the levels are indistinguishable in the catalog
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>see the proposed description above</t>
           </r>
         </is>
       </c>
@@ -2010,16 +1975,35 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Perform major and minor scales and arpeggios across Group 1 and Group 2 keys, two octaves. 2. Play triads in all inversions and perform the dominant seventh chord in block and broken patterns. 3. Harmonize short melodies using primary chords (I, IV, V⁷) in major and minor, with idiomatic accompaniment patterns including Alberti and waltz bass. 4. Sing a melody while playing a two-hand accompaniment. 5. Realize basic lead-sheet symbols and Roman numerals at the keyboard. 6. Sight-read in grand staff, hands together, in four-to-eight-bar examples.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Second of three concurrent keyboard courses for music majors. Major and minor scales and arpeggios across the first two key groups, primary chords in block and broken patterns, melodic harmonization, lead-sheet realization, and hands-together sight-reading.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to the other courses in its track, so the levels are indistinguishable in the catalog
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>see the proposed description above</t>
           </r>
         </is>
       </c>
@@ -2283,7 +2267,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">classified C09 large group where MUS 111 and MUS 112 are C10 small group → </t>
+            <t xml:space="preserve">classified C09 large group where MUS 111 and MUS 112 are C10 small group
+</t>
           </r>
           <r>
             <rPr>
@@ -2296,50 +2281,7 @@
           </r>
         </is>
       </c>
-      <c r="U18" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>The last of three intensive courses that introduce students to the inner workings of European art music of the 18th and 19th centuries. This course covers chromatic harmony, tonicization and modulation, and other advanced tonal procedures.</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Write and analyze chromatic harmony, including applied dominants, modal mixture, the Neapolitan sixth, augmented sixth chords, and altered chords. 2. Identify and compose modulations to the dominant and to closely related keys. 3. Analyze chromatic sequences and chromatic modulation. 4. Evaluate tonal works combining diatonic and chromatic vocabulary in extended harmonic contexts. 5. Apply chromatic harmonic vocabulary at the keyboard and in performance on the student's primary instrument or voice.</t>
-          </r>
-        </is>
-      </c>
+      <c r="U18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2425,7 +2367,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-10, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-10, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -2445,16 +2388,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Sing and hear harmonically, following harmonic rhythm and cadences. 2. Work in two-voice textures and take bass-line dictation. 3. Identify root-position and first-inversion triads and all four triad qualities by ear, and sing melodic skips through every diatonic triad (leading-tone, supertonic, submediant, and mediant). 4. Handle the dominant seventh chord in harmonic context, with the voice-leading techniques that close the lower-division sequence.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Third of three concurrent aural skills courses. Harmonic listening and dictation: harmonic rhythm and cadences, two-voice textures, bass-line dictation, triad quality and inversion by ear, and melodic skips through every diatonic triad.</t>
           </r>
         </is>
       </c>
@@ -2544,16 +2488,35 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Perform major and minor scales and arpeggios across all key groups, and play chromatic, whole-tone, and blues scales. 2. Perform secondary triads (ii, iii, vi) and seventh chords in harmonic context, with correct voice leading. 3. Play melodies and accompaniments in all six church modes. 4. Harmonize melodies using the full diatonic vocabulary including secondary chords. 5. Transpose short examples to other keys and improvise within defined modal and harmonic frameworks. 6. Prepare and perform repertoire from Alfred's Book 1 for peers and instructor.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Third of three concurrent keyboard courses for music majors. Scales and arpeggios in all key groups, secondary triads and seventh chords in harmonic context, chromatic, whole-tone, and blues scales, and playing in all six church modes.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to the other courses in its track, so the levels are indistinguishable in the catalog
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>see the proposed description above</t>
           </r>
         </is>
       </c>
@@ -2922,7 +2885,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-01, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-01, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -3014,7 +2978,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-01, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-01, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -3194,7 +3159,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the individual lower division applied norm is 8 → </t>
+            <t xml:space="preserve">repeat cap of 4 units where the individual lower division applied norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -3214,7 +3180,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -3317,7 +3284,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of MUS 111 where MUS 262G and MUS 263G require none → </t>
+            <t xml:space="preserve">prerequisite of MUS 111 where MUS 262G and MUS 263G require none
+</t>
           </r>
           <r>
             <rPr>
@@ -3417,7 +3385,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -3516,7 +3485,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes 1 and 2 are merged into a single numbered item → </t>
+            <t xml:space="preserve">outcomes 1 and 2 are merged into a single numbered item
+</t>
           </r>
           <r>
             <rPr>
@@ -3614,7 +3584,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 46 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 46 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -3634,7 +3605,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -3650,15 +3622,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcome 3 names the violin in a course covering violin, viola, cello, bass, guitar, and harp → </t>
+            <t xml:space="preserve">
+outcome 3 names the violin in a course covering violin, viola, cello, bass, guitar, and harp
+</t>
           </r>
           <r>
             <rPr>
@@ -3837,7 +3803,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 45 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 45 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -3857,7 +3824,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -3873,15 +3841,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcome 3 names the flute in a course covering flute, clarinet, oboe, bassoon, and saxophone → </t>
+            <t xml:space="preserve">
+outcome 3 names the flute in a course covering flute, clarinet, oboe, bassoon, and saxophone
+</t>
           </r>
           <r>
             <rPr>
@@ -3979,7 +3941,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -4077,7 +4040,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the individual lower division applied norm is 8 → </t>
+            <t xml:space="preserve">repeat cap of 4 units where the individual lower division applied norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -4097,7 +4061,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -4278,7 +4243,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-09, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-09, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -4294,15 +4260,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">classified S36 where other studio courses are C36 → </t>
+            <t xml:space="preserve">
+classified S36 where other studio courses are C36
+</t>
           </r>
           <r>
             <rPr>
@@ -4318,48 +4278,36 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">fixed at 1 unit, so a junior or senior recitalist cannot enroll in the 2 units the handbook requires in the recital semester → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1-2</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add the credit restriction: Units may not be used towards the Music Major or Minor.</t>
+            <t xml:space="preserve">
+fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set units to 1–2</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add: Units may not be used towards the Music Major or Minor.</t>
           </r>
         </is>
       </c>
@@ -4370,7 +4318,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -4386,15 +4335,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes are the generic applied study set and outcome 2 addresses tone production on the primary instrument → </t>
+            <t xml:space="preserve">
+outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
+</t>
           </r>
           <r>
             <rPr>
@@ -4496,7 +4439,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-09, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-09, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -4512,15 +4456,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">classified S36 where other studio courses are C36 → </t>
+            <t xml:space="preserve">
+classified S36 where other studio courses are C36
+</t>
           </r>
           <r>
             <rPr>
@@ -4536,48 +4474,36 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">fixed at 1 unit, so a junior or senior recitalist cannot enroll in the 2 units the handbook requires in the recital semester → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1-2</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add the credit restriction: Units may not be used towards the Music Major or Minor.</t>
+            <t xml:space="preserve">
+fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set units to 1–2</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add: Units may not be used towards the Music Major or Minor.</t>
           </r>
         </is>
       </c>
@@ -4588,7 +4514,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -4604,15 +4531,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes are the generic applied study set and outcome 2 addresses tone production on the primary instrument → </t>
+            <t xml:space="preserve">
+outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
+</t>
           </r>
           <r>
             <rPr>
@@ -5071,7 +4992,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 43 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 43 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -5087,15 +5009,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">reclassification pending per the theory and musicianship guide, effective fall 2027 → </t>
+            <t xml:space="preserve">
+reclassification pending per the theory and musicianship guide, effective fall 2027
+</t>
           </r>
           <r>
             <rPr>
@@ -5115,7 +5031,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -5125,30 +5042,6 @@
               <sz val="10"/>
             </rPr>
             <t>Analysis of style and structural form in European art music of the 18th and 19th centuries. Topics include phrase and sentence structure, thematic organization, binary and ternary forms, variation and rondo forms, slow movement forms, and sonata forms.</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Demonstrate understanding of the forms used in tonal music, including sentence, period, binary, ternary, rondo, and sonata forms. 2. Analyze and evaluate complete tonal works in their technical, aesthetic, and historical contexts, supporting interpretive claims with evidence from the score. 3. Apply the harmonic and contrapuntal knowledge of the lower-division sequence to extended musical works. 4. Identify phrase structure, hypermeter, and formal boundaries both visually and aurally. 5. Construct written analyses using appropriate terminology, Roman numerals, figured bass, and formal labels. 6. Implement the principles and concepts studied in class via performance on the student's major instrument or voice.</t>
           </r>
         </is>
       </c>
@@ -5235,7 +5128,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 42 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 42 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -5255,7 +5149,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -5568,7 +5463,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -5656,7 +5552,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published → </t>
+            <t xml:space="preserve">no learning outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -5672,15 +5569,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">
+repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -5700,7 +5591,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published → </t>
+            <t xml:space="preserve">no outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -5792,7 +5684,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -5808,15 +5701,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-18, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-02-18, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -5908,7 +5795,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -6003,7 +5891,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 3 where the record holds 2 → </t>
+            <t xml:space="preserve">units publish as 3 where the record holds 2
+</t>
           </r>
           <r>
             <rPr>
@@ -6019,15 +5908,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-04-26, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-04-26, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -6043,15 +5926,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 3 where the record holds 2 → </t>
+            <t xml:space="preserve">
+units publish as 3 where the record holds 2
+</t>
           </r>
           <r>
             <rPr>
@@ -6148,7 +6025,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -6246,7 +6124,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -6346,7 +6225,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">title published as Band: Wind Ensemble where the handbook names the ensemble East Bay Wind Symphony → </t>
+            <t xml:space="preserve">title published as Band: Wind Ensemble where the handbook names the ensemble East Bay Wind Symphony
+</t>
           </r>
           <r>
             <rPr>
@@ -6366,7 +6246,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -6465,7 +6346,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -6560,7 +6442,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -6580,7 +6463,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -6679,7 +6563,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -6695,15 +6580,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">grading A-F or CR/NC (student choice) where the chamber ensemble norm is A-F or CR/NC (student choice) → </t>
+            <t xml:space="preserve">
+grading A-F or CR/NC (student choice) where the chamber ensemble norm is A-F or CR/NC (student choice)
+</t>
           </r>
           <r>
             <rPr>
@@ -6798,7 +6677,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeat cap of 6 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">repeat cap of 6 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -6814,15 +6694,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice) → </t>
+            <t xml:space="preserve">
+grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice)
+</t>
           </r>
           <r>
             <rPr>
@@ -6842,7 +6716,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -6936,7 +6811,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-12, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-12, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -6952,15 +6828,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">
+repeat cap of 4 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -6976,15 +6846,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice) → </t>
+            <t xml:space="preserve">
+grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice)
+</t>
           </r>
           <r>
             <rPr>
@@ -7004,7 +6868,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7098,7 +6963,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice) → </t>
+            <t xml:space="preserve">grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice)
+</t>
           </r>
           <r>
             <rPr>
@@ -7118,7 +6984,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7212,7 +7079,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 41 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 41 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -7228,15 +7096,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">
+repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -7256,7 +7118,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7352,7 +7215,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-12, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-12, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -7368,15 +7232,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">
+repeat cap of 4 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -7396,7 +7254,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7492,7 +7351,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeat cap of 6 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">repeat cap of 6 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -7508,15 +7368,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice) → </t>
+            <t xml:space="preserve">
+grading A-F grading only where the chamber ensemble norm is A-F or CR/NC (student choice)
+</t>
           </r>
           <r>
             <rPr>
@@ -7536,7 +7390,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7633,7 +7488,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-19, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-19, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -7649,15 +7505,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">
+repeat cap of 4 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -7677,7 +7527,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7773,7 +7624,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-19, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-19, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -7789,15 +7641,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">
+repeat cap of 4 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -7817,7 +7663,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -7910,7 +7757,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeat cap of 4 units where the chamber ensemble norm is 8 → </t>
+            <t xml:space="preserve">repeat cap of 4 units where the chamber ensemble norm is 8
+</t>
           </r>
           <r>
             <rPr>
@@ -7926,15 +7774,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">title published as Jazz Singers where the handbook names the ensemble East Bay Jazz Singers → </t>
+            <t xml:space="preserve">
+title published as Jazz Singers where the handbook names the ensemble East Bay Jazz Singers
+</t>
           </r>
           <r>
             <rPr>
@@ -7954,7 +7796,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -8051,7 +7894,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -8218,7 +8062,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -8309,7 +8154,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">reclassification pending per the theory and musicianship guide, effective fall 2027 → </t>
+            <t xml:space="preserve">reclassification pending per the theory and musicianship guide, effective fall 2027
+</t>
           </r>
           <r>
             <rPr>
@@ -8329,16 +8175,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes, from the syllabus → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Demonstrate understanding of the different genres, styles, and techniques of 20th and 21st century art music. 2. Analyze and evaluate post-tonal works in their technical, aesthetic, and historical contexts, supporting interpretive claims with evidence from the score. 3. Construct and manipulate post-tonal pitch collections, including pitch-class sets in normal and prime form, and analyze twelve-tone rows and their transformations. 4. Apply knowledge from earlier theory courses to extended post-tonal and contemporary works. 5. Situate works within the major compositional movements of the 20th and 21st centuries, including serialism, spectralism, minimalism, and extended techniques. 6. Implement the principles and concepts studied in class via performance on the student's area of emphasis.</t>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Analytical and compositional techniques of the 20th and 21st centuries: post-tonal collections, pitch-class sets, centricity, twelve-tone serialism, form in post-tonal music, and the movements that follow 1945, including spectralism and minimalism.</t>
           </r>
         </is>
       </c>
@@ -8650,7 +8497,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -8749,7 +8597,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -8845,7 +8694,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -8945,7 +8795,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 3 where the record holds 2 → </t>
+            <t xml:space="preserve">units publish as 3 where the record holds 2
+</t>
           </r>
           <r>
             <rPr>
@@ -8961,15 +8812,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-04-27, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-04-27, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -8985,15 +8830,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 3 where the record holds 2 → </t>
+            <t xml:space="preserve">
+units publish as 3 where the record holds 2
+</t>
           </r>
           <r>
             <rPr>
@@ -9169,7 +9008,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -9272,7 +9112,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 261A, renumbered or discontinued → </t>
+            <t xml:space="preserve">requires MUS 261A, renumbered or discontinued
+</t>
           </r>
           <r>
             <rPr>
@@ -9292,7 +9133,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -9308,15 +9150,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">
+outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -9419,7 +9255,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -9522,7 +9359,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -9538,15 +9376,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">
+outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -9649,7 +9481,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -9747,7 +9580,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite ends with a doubled period → </t>
+            <t xml:space="preserve">prerequisite ends with a doubled period
+</t>
           </r>
           <r>
             <rPr>
@@ -9767,7 +9601,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -9870,7 +9705,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -9973,7 +9809,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10076,7 +9913,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10174,7 +10012,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes 1 and 2 are merged into a single numbered item → </t>
+            <t xml:space="preserve">outcomes 1 and 2 are merged into a single numbered item
+</t>
           </r>
           <r>
             <rPr>
@@ -10190,15 +10029,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">
+outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10301,7 +10134,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10404,7 +10238,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10506,7 +10341,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 180, renumbered or discontinued → </t>
+            <t xml:space="preserve">requires MUS 180, renumbered or discontinued
+</t>
           </r>
           <r>
             <rPr>
@@ -10522,15 +10358,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">prerequisite written without a space in the course number → </t>
+            <t xml:space="preserve">
+prerequisite written without a space in the course number
+</t>
           </r>
           <r>
             <rPr>
@@ -10550,7 +10380,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10652,7 +10483,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 180, renumbered or discontinued → </t>
+            <t xml:space="preserve">requires MUS 180, renumbered or discontinued
+</t>
           </r>
           <r>
             <rPr>
@@ -10668,15 +10500,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">prerequisite written without a space in the course number → </t>
+            <t xml:space="preserve">
+prerequisite written without a space in the course number
+</t>
           </r>
           <r>
             <rPr>
@@ -10696,7 +10522,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10798,7 +10625,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite written without a space in the course number → </t>
+            <t xml:space="preserve">prerequisite written without a space in the course number
+</t>
           </r>
           <r>
             <rPr>
@@ -10818,7 +10646,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person → </t>
+            <t xml:space="preserve">outcome 3 reads creating new repertoire and addresses the student in the second person, where the lower division series reads learning new repertoire in the third person
+</t>
           </r>
           <r>
             <rPr>
@@ -10920,16 +10749,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add the credit restriction: Units may not be used towards the Music Major or Minor.</t>
+            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add: Units may not be used towards the Music Major or Minor.</t>
           </r>
         </is>
       </c>
@@ -10940,7 +10770,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -10956,15 +10787,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes are the generic applied study set and outcome 2 addresses tone production on the primary instrument → </t>
+            <t xml:space="preserve">
+outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
+</t>
           </r>
           <r>
             <rPr>
@@ -11066,16 +10891,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add the credit restriction: Units may not be used towards the Music Major or Minor.</t>
+            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add: Units may not be used towards the Music Major or Minor.</t>
           </r>
         </is>
       </c>
@@ -11086,7 +10912,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -11102,15 +10929,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">outcomes are the generic applied study set and outcome 2 addresses tone production on the primary instrument → </t>
+            <t xml:space="preserve">
+outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
+</t>
           </r>
           <r>
             <rPr>
@@ -11357,7 +11178,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published → </t>
+            <t xml:space="preserve">no learning outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -11373,15 +11195,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">
+no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -11401,7 +11217,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published → </t>
+            <t xml:space="preserve">no outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -11500,7 +11317,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1 where the record holds 2 → </t>
+            <t xml:space="preserve">units publish as 1 where the record holds 2
+</t>
           </r>
           <r>
             <rPr>
@@ -11516,15 +11334,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-05-13, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-05-13, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -11540,15 +11352,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 2 where the music education certificate roadmap and handbook give 1 → </t>
+            <t xml:space="preserve">
+units publish as 2 where the certificate roadmap and handbook give 1
+</t>
           </r>
           <r>
             <rPr>
@@ -11639,7 +11445,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-01, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">last revised 2016-05-01, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -11960,7 +11767,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1-3 where the record holds 1 → </t>
+            <t xml:space="preserve">units publish as 1-3 where the record holds 1
+</t>
           </r>
           <r>
             <rPr>
@@ -11976,24 +11784,18 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">record holds 1 unit where the catalog and handbook give 1-3 → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>correct the record to 1-3</t>
+            <t xml:space="preserve">
+record holds 1 unit where the catalog and handbook give 1–3
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>correct the record to 1–3</t>
           </r>
         </is>
       </c>
@@ -12080,7 +11882,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -12096,15 +11899,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-05, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-02-05, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -12702,7 +12499,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -12718,15 +12516,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-24, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-02-24, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -12981,7 +12773,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -13073,7 +12866,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -13172,7 +12966,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses → </t>
+            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+</t>
           </r>
           <r>
             <rPr>
@@ -13270,7 +13065,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 669, renumbered or discontinued → </t>
+            <t xml:space="preserve">requires MUS 669, renumbered or discontinued
+</t>
           </r>
           <r>
             <rPr>
@@ -13286,15 +13082,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses → </t>
+            <t xml:space="preserve">
+prerequisite of department consent, absent on most graduate applied courses
+</t>
           </r>
           <r>
             <rPr>
@@ -13392,7 +13182,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses → </t>
+            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+</t>
           </r>
           <r>
             <rPr>
@@ -13491,7 +13282,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses → </t>
+            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+</t>
           </r>
           <r>
             <rPr>
@@ -13586,7 +13378,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 41 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 41 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -13606,7 +13399,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -13923,7 +13717,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1 where the record holds 1-2 → </t>
+            <t xml:space="preserve">units publish as 1 where the record holds 1-2
+</t>
           </r>
           <r>
             <rPr>
@@ -13939,24 +13734,18 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 1 where the other graduate applied courses publish 1-2 → </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1-2</t>
+            <t xml:space="preserve">
+units publish as 1 where the other graduate applied courses publish 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set units to 1–2</t>
           </r>
         </is>
       </c>
@@ -14273,7 +14062,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses → </t>
+            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+</t>
           </r>
           <r>
             <rPr>
@@ -14517,7 +14307,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published → </t>
+            <t xml:space="preserve">no learning outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -14533,15 +14324,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">
+repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -14561,7 +14346,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published → </t>
+            <t xml:space="preserve">no outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -14660,7 +14446,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -14752,7 +14539,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published → </t>
+            <t xml:space="preserve">no learning outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -14768,15 +14556,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing → </t>
+            <t xml:space="preserve">
+repeatability uses non-standard phrasing
+</t>
           </r>
           <r>
             <rPr>
@@ -14796,7 +14578,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published → </t>
+            <t xml:space="preserve">no outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -14883,7 +14666,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published → </t>
+            <t xml:space="preserve">no learning outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -14899,15 +14683,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">
+no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -14923,15 +14701,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-26, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-02-26, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -14951,7 +14723,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published → </t>
+            <t xml:space="preserve">no outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -15044,7 +14817,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 42 words, over the 40-word limit → </t>
+            <t xml:space="preserve">description runs to 42 words, over the 40-word limit
+</t>
           </r>
           <r>
             <rPr>
@@ -15060,15 +14834,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">
+no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -15084,15 +14852,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-26, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-02-26, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -15112,7 +14874,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description → </t>
+            <t xml:space="preserve">description
+</t>
           </r>
           <r>
             <rPr>
@@ -15205,7 +14968,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1-6 where the record holds 6 → </t>
+            <t xml:space="preserve">units publish as 1-6 where the record holds 6
+</t>
           </r>
           <r>
             <rPr>
@@ -15374,7 +15138,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -15390,15 +15155,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-26, still on the 2016 conversion form → </t>
+            <t xml:space="preserve">
+last revised 2016-02-26, still on the 2016 conversion form
+</t>
           </r>
           <r>
             <rPr>
@@ -15486,7 +15245,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published → </t>
+            <t xml:space="preserve">no learning outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -15502,15 +15262,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no teaching component or classification on record → </t>
+            <t xml:space="preserve">
+no teaching component or classification on record
+</t>
           </r>
           <r>
             <rPr>
@@ -15526,15 +15280,9 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no proposal on record in the Curriculog archive → </t>
+            <t xml:space="preserve">
+no proposal on record in the Curriculog archive
+</t>
           </r>
           <r>
             <rPr>
@@ -15554,7 +15302,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published → </t>
+            <t xml:space="preserve">no outcomes published
+</t>
           </r>
           <r>
             <rPr>
@@ -15648,7 +15397,8 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1-6 where the record holds 6 → </t>
+            <t xml:space="preserve">units publish as 1-6 where the record holds 6
+</t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Source the sequence findings from the repo files
The workbook now reads the proposed descriptions, outcomes, and
requisites for the twelve sequence courses out of the syllabi and the
guide rather than holding its own copy, so the audit and the repo
cannot drift apart.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1401,6 +1401,24 @@
               <color rgb="00B03A2E"/>
               <sz val="10"/>
             </rPr>
+            <t>prerequisite: MUS 108, or satisfactory score on the Music Theory Advisory Exam, or department consent</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+corequisite carries no equivalence or consent path
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
             <t>corequisite: MUS 115 and MUS 118, or equivalent, or department consent</t>
           </r>
         </is>
@@ -1547,17 +1565,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-strongly recommended preparation duplicates the proposed prerequisite
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>remove the strongly recommended preparation, now covered by the prerequisite</t>
+strongly recommended preparation duplicates the prerequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the strongly recommended preparation</t>
           </r>
         </is>
       </c>
@@ -1568,7 +1586,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes repeat the closing three of MUS 111 and MUS 211 and name no level-specific content, where the syllabus outcomes from the musicianship overhaul are current
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The second of three intensive courses that introduce students to the inner workings of European art music of the 18th and 19th centuries. This course completes diatonic harmony and introduces advanced part-writing, voice-leading, and harmonization techniques.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+outcomes repeat the closing three of MUS 111 and MUS 211 and name no level-specific content, where the syllabus outcomes from the musicianship overhaul are current
 </t>
           </r>
           <r>
@@ -2513,17 +2549,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-strongly recommended preparation duplicates the proposed prerequisite
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>remove the strongly recommended preparation, now covered by the prerequisite</t>
+strongly recommended preparation duplicates the prerequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the strongly recommended preparation</t>
           </r>
         </is>
       </c>
@@ -2651,17 +2687,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-corequisite carries no equivalence or consent path for transfer students
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>prerequisite: MUS 112 and MUS 116, or equivalent, or department consent</t>
+prerequisite and corequisite differ from the syllabus and carry no equivalence or consent path
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>prerequisite: MUS 116, or equivalent, or department consent</t>
           </r>
           <r>
             <rPr>
@@ -2679,7 +2715,7 @@
               <color rgb="00B03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>corequisite: MUS 211, or equivalent, or department consent</t>
+            <t>corequisite: MUS 211 and MUS 218, or equivalent, or department consent</t>
           </r>
         </is>
       </c>
@@ -5386,17 +5422,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-prerequisite misspells successful
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>correct to: MUS 211, or successful Theory and Musicianship Placement Exam</t>
+prerequisite misspells successful and names only MUS 211
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>prerequisite: MUS 211, MUS 215, and MUS 218, or successful Theory and Musicianship Placement Exam, or department consent</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Add credit by exam to MUS 118
Students may test out of Keyboard I outright, which the handbook
supports with a credit-by-exam guide for all three levels. MUS 118
now carries that route alongside its corequisites.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -2026,7 +2026,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no corequisite published, though the guide runs the three tracks concurrently
+            <t xml:space="preserve">no requisites published, though the guide runs the three tracks concurrently and the handbook offers credit by exam
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>prerequisite: None; credit by exam available</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+corequisite carries no equivalence or consent path
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
Drop credit by exam from the keyboard requisites
Credit by exam is a route around a requirement rather than a way of
satisfying a prerequisite, so it does not belong in the requisite
fields. The keyboard courses now read the course, or equivalent, or
department consent, matching the rest of the sequence. Credit by exam
remains documented in the undergraduate handbook.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -2026,25 +2026,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no requisites published, though the guide runs the three tracks concurrently and the handbook offers credit by exam
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>prerequisite: None; credit by exam available</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-corequisite carries no equivalence or consent path
+            <t xml:space="preserve">no corequisite published, though the guide runs the three tracks concurrently
 </t>
           </r>
           <r>
@@ -2192,7 +2174,7 @@
               <color rgb="00B03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>prerequisite: MUS 118, or equivalent, or credit by exam</t>
+            <t>prerequisite: MUS 118, or equivalent, or department consent</t>
           </r>
           <r>
             <rPr>
@@ -2871,7 +2853,7 @@
               <color rgb="00B03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>prerequisite: MUS 119, or equivalent, or credit by exam</t>
+            <t>prerequisite: MUS 119, or equivalent, or department consent</t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Correct the MUS 495 unit finding in the course inventory
The technical findings for MUS 495 carried two statements that
contradicted each other on which unit value the catalog publishes.
The catalog publishes 1 unit. Removed the block asserting that it
publishes 2.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -11813,24 +11813,6 @@
             </rPr>
             <t>review the full record on the current form</t>
           </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-units publish as 2 where the certificate roadmap and handbook give 1
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1</t>
-          </r>
         </is>
       </c>
       <c r="U101" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Correct the MUS 441 unit finding to name the classification as stale
The published 3 units are correct. The record's C05 2u is a quarter-to-
semester conversion artifact from the 2016 form. The finding now calls for
the classification to be set to C05 3u rather than for published units to
be changed to 3, and the duplicated entry is consolidated.

MUS 441 in the spring 2027 slate moves to 3.0 WTU. Music education subtotal
7.3, total 51.9.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -9259,24 +9259,21 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 3 where the record holds 2
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 3</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification holds 2 units of C05 where the course publishes 3, a quarter-conversion artifact
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+            </rPr>
+            <t>set the classification to C05 3u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
             </rPr>
             <t xml:space="preserve">
 last revised 2016-04-27, still on the 2016 conversion form
@@ -9287,27 +9284,8 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00B03A2E"/>
-              <sz val="10"/>
             </rPr>
             <t>review the full record on the current form</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-units publish as 3 where the record holds 2
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>correct the record to 3</t>
           </r>
         </is>
       </c>
@@ -15864,8 +15842,5 @@
   </sheetData>
   <autoFilter ref="A1:U141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:U141" numberStoredAsText="1" twoDigitTextYear="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Close the spring 2027 open items and file the MUS 693 classification
MUS 693 is S25, supervision, at .48 WTU per student. Recorded in the
graduate studies section of the slate, and the audit now carries a finding
to set the classification from C25 to S25.

The remaining open items are resolved and the section is removed:
corequisites are handled with codes pending the revisions, MUS 410 runs at
C02 for 3.0 this term, MUS 414 is the composition course, and MUS 365 stays
at C10.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -15482,7 +15482,25 @@
       <c r="S138" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="T138" s="3" t="inlineStr"/>
+      <c r="T138" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+            </rPr>
+            <t xml:space="preserve">classified C25, which is not a CSUEB course classification
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+            </rPr>
+            <t>set the classification to S25</t>
+          </r>
+        </is>
+      </c>
       <c r="U138" s="3" t="inlineStr"/>
     </row>
     <row r="139">

</xml_diff>

<commit_message>
Correct the MUS 341 unit finding to match MUS 441
MUS 341 Basic Conducting publishes 3 units against a record of C05 2u from
the 2016 conversion form, the same quarter-to-semester artifact as MUS 441.
The finding now calls for the classification to be set to C05 3u.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -6319,24 +6319,21 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 3 where the record holds 2
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 3</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification holds 2 units of C05 where the course publishes 3, a quarter-conversion artifact
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00B03A2E"/>
+            </rPr>
+            <t>set the classification to C05 3u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
             </rPr>
             <t xml:space="preserve">
 last revised 2016-04-26, still on the 2016 conversion form
@@ -6347,27 +6344,8 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00B03A2E"/>
-              <sz val="10"/>
             </rPr>
             <t>review the full record on the current form</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-units publish as 3 where the record holds 2
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00B03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>correct the record to 3</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Mark the courses to discontinue and to bank
The findings are replaced with the intended action on the seven marked
rows. Discontinue: MUS 691, 692, 699. Bank: MUS 671, 676, 678, 697. The
content findings on those rows are cleared.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -6768,19 +6768,11 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 4 units</t>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>bank</t>
           </r>
         </is>
       </c>
@@ -6858,61 +6850,15 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no learning outcomes published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 4 units</t>
-          </r>
-        </is>
-      </c>
-      <c r="T60" s="7" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no outcomes published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>to be drafted by area faculty</t>
-          </r>
-        </is>
-      </c>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>bank</t>
+          </r>
+        </is>
+      </c>
+      <c r="T60" s="7" t="n"/>
     </row>
     <row r="61" ht="112" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
@@ -7112,61 +7058,15 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description runs to 42 words, over the 40-word limit
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>shorten to 40 words or fewer</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-last revised 2016-02-26, still on the 2016 conversion form
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>review the full record on the current form</t>
-          </r>
-        </is>
-      </c>
-      <c r="T62" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Development and completion of a formal written thesis for submission to the university. Supervision by a departmental committee, at least one member of which must be a Cal State East Bay faculty member. Oral defense required.</t>
-          </r>
-        </is>
-      </c>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>discontinue</t>
+          </r>
+        </is>
+      </c>
+      <c r="T62" s="9" t="n"/>
     </row>
     <row r="63" ht="112" customHeight="1">
       <c r="A63" s="8" t="inlineStr">
@@ -7242,19 +7142,11 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 1-6 where the record holds 6
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1-6</t>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>discontinue</t>
           </r>
         </is>
       </c>
@@ -7426,19 +7318,11 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">last revised 2016-02-26, still on the 2016 conversion form
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>review the full record on the current form</t>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>bank</t>
           </r>
         </is>
       </c>
@@ -7643,19 +7527,11 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">units publish as 1-6 where the record holds 6
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1-6</t>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>discontinue</t>
           </r>
         </is>
       </c>
@@ -15530,61 +15406,15 @@
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no learning outcomes published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 4 units</t>
-          </r>
-        </is>
-      </c>
-      <c r="T23" s="7" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">no outcomes published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>to be drafted by area faculty</t>
-          </r>
-        </is>
-      </c>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>bank</t>
+          </r>
+        </is>
+      </c>
+      <c r="T23" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:T23"/>

</xml_diff>

<commit_message>
Drop the repeatability phrasing finding
The finding is removed from all seven courses that carried it. Four now
carry no technical finding: MUS 109, 110, 351A, 360. Three keep their
remaining findings: MUS 326, 360A, 366.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1157,27 +1157,7 @@
           <t>2023-09-14</t>
         </is>
       </c>
-      <c r="S8" s="3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 6 units</t>
-          </r>
-        </is>
-      </c>
+      <c r="S8" s="3" t="n"/>
       <c r="T8" s="2" t="n"/>
     </row>
     <row r="9">
@@ -1250,27 +1230,7 @@
           <t>2023-09-14</t>
         </is>
       </c>
-      <c r="S9" s="3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 3 units</t>
-          </r>
-        </is>
-      </c>
+      <c r="S9" s="3" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
     <row r="10" ht="126" customHeight="1">
@@ -4310,24 +4270,6 @@
               <sz val="10"/>
             </rPr>
             <t>add learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 9 units</t>
           </r>
         </is>
       </c>
@@ -11546,27 +11488,7 @@
           <t>2025-09-14</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 8 units</t>
-          </r>
-        </is>
-      </c>
+      <c r="S2" s="3" t="n"/>
       <c r="T2" s="2" t="n"/>
     </row>
     <row r="3">
@@ -11951,27 +11873,7 @@
           <t>2023-02-14</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 8 units</t>
-          </r>
-        </is>
-      </c>
+      <c r="S6" s="3" t="n"/>
       <c r="T6" s="3" t="inlineStr">
         <is>
           <r>
@@ -12076,25 +11978,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 8 units</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-grading A-F or CR/NC (student choice) where the chamber ensemble norm is A-F or CR/NC (student choice)
+            <t xml:space="preserve">grading A-F or CR/NC (student choice) where the chamber ensemble norm is A-F or CR/NC (student choice)
 </t>
           </r>
           <r>
@@ -12591,24 +12475,6 @@
               <sz val="10"/>
             </rPr>
             <t>shorten to 40 words or fewer</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeatability uses non-standard phrasing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reword to may be repeated for credit for a maximum of 8 units</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Add the MUS 324 outcomes finding and the C36 unit rule
MUS 324 holds the three Diversity Overlay outcomes in the course learning
outcomes column and publishes no course outcomes. The catalog audit README
records that a 1-2 unit range against a C36 1u classification is correct:
each unit carries the classification.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4259,7 +4259,27 @@
           <t>2020-10-06</t>
         </is>
       </c>
-      <c r="S33" s="5" t="n"/>
+      <c r="S33" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">the three Diversity Overlay outcomes sit in the course learning outcomes, and no course outcomes are published
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add course learning outcomes and hold the overlay outcomes as breadth outcomes</t>
+          </r>
+        </is>
+      </c>
       <c r="T33" s="4" t="n"/>
     </row>
     <row r="34" ht="70" customHeight="1" s="12">

</xml_diff>

<commit_message>
Standardize the coaching series and revise the two internships
The six coaching courses carry matching findings: 1-2 units, C36 1u, and a
16-unit repeat cap, with proposed descriptions and learning outcomes that
separate vocal from instrumental and lower division from upper division.
MUS 660A and 660B keep their existing outcomes.

The credit restriction that keeps coaching units off the major and minor is
dropped from MUS 281, 282, 481, and 482, and MUS 498 carries a finding to
remove the one it publishes.

MUS 498 and MUS 698 carry proposed descriptions and learning outcomes. The
MUS 698 row is wrapped.

The issue lines on MUS 111, 116, 211, and 215 name the field their change
alters.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1364,7 +1364,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">corequisite carries no equivalence or consent path for transfer students
+            <t xml:space="preserve">prerequisite names the Music Theory Advisory Exam, no longer administered, and carries no equivalence or consent path
 </t>
           </r>
           <r>
@@ -1837,7 +1837,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-corequisite names MUS 118B, renumbered to MUS 119 in September 2019
+prerequisite carries no equivalence or consent path
 </t>
           </r>
           <r>
@@ -1855,7 +1855,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-corequisite carries no equivalence or consent path
+corequisite names MUS 118B, renumbered to MUS 119 in September 2019, and carries no equivalence or consent path
 </t>
           </r>
           <r>
@@ -2462,7 +2462,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-corequisite carries no equivalence or consent path for transfer students
+prerequisite carries no equivalence or consent path for transfer students
 </t>
           </r>
           <r>
@@ -2633,7 +2633,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-prerequisite and corequisite differ from the syllabus and carry no equivalence or consent path
+prerequisite names MUS 112 and MUS 116 where the syllabus names MUS 116, and carries no equivalence or consent path
 </t>
           </r>
           <r>
@@ -3019,17 +3019,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-09, still on the 2016 conversion form
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>review the full record on the current form</t>
+            <t xml:space="preserve">fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set units to 1–2</t>
           </r>
           <r>
             <rPr>
@@ -3037,17 +3037,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-classified S36 where other studio courses are C36
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reclassify to C36</t>
+classified S36 where the rest of the coaching series is C36
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>reclassify to C36 1u</t>
           </r>
           <r>
             <rPr>
@@ -3055,17 +3055,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1–2</t>
+description is identical to MUS 481 and carries no level marker
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
           </r>
           <r>
             <rPr>
@@ -3073,17 +3073,35 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add: Units may not be used towards the Music Major or Minor.</t>
+learning outcomes are identical to MUS 282, MUS 481, and MUS 482, are written for applied study, and name the primary instrument on a vocal course
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+repeat cap differs across the coaching series
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -3104,7 +3122,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>Individual coaching with a faculty coach on repertoire requiring a collaborative pianist, for students enrolled in applied study. Coaching times are arranged according to degree recital expectations. Requirements appear in the Music Student Handbook.</t>
+            <t>Individual vocal coaching with a collaborative pianist for music majors and minors at the lower division performance level. Coaching times arranged according to the expectations in the Music Student Handbook.</t>
           </r>
           <r>
             <rPr>
@@ -3112,17 +3130,20 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Prepare repertoire with a collaborative pianist to a performance standard. 2. Apply rehearsal technique to balance, ensemble coordination, and pacing with a collaborator. 3. Communicate interpretive decisions clearly to collaborating musicians. 4. Perform prepared repertoire with a collaborative pianist in juries and recitals.</t>
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Prepare vocal repertoire with a collaborative pianist, marking and rehearsing entrances, cutoffs, tempo, and balance.
+2. Apply diction and text translation to the delivery of the repertoire.
+3. Rehearse and perform with a collaborative pianist, responding to the accompaniment in the moment.
+4. Document the preparation of a work from first rehearsal to performance.</t>
           </r>
         </is>
       </c>
@@ -3212,17 +3233,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">last revised 2016-05-09, still on the 2016 conversion form
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>review the full record on the current form</t>
+            <t xml:space="preserve">fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set units to 1–2</t>
           </r>
           <r>
             <rPr>
@@ -3230,17 +3251,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-classified S36 where other studio courses are C36
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reclassify to C36</t>
+classified S36 where the rest of the coaching series is C36
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>reclassify to C36 1u</t>
           </r>
           <r>
             <rPr>
@@ -3248,17 +3269,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1–2</t>
+description is identical to MUS 482 and carries no level marker
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
           </r>
           <r>
             <rPr>
@@ -3266,17 +3287,35 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add: Units may not be used towards the Music Major or Minor.</t>
+learning outcomes are identical to MUS 281, MUS 481, and MUS 482 and are written for applied study
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+repeat cap differs across the coaching series
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -3297,7 +3336,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>Individual coaching with a faculty coach on repertoire requiring a collaborative pianist, for students enrolled in applied study. Coaching times are arranged according to degree recital expectations. Requirements appear in the Music Student Handbook.</t>
+            <t>Individual instrumental coaching with a collaborative pianist for music majors and minors at the lower division performance level. Coaching times arranged according to the expectations in the Music Student Handbook.</t>
           </r>
           <r>
             <rPr>
@@ -3305,17 +3344,20 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Prepare repertoire with a collaborative pianist to a performance standard. 2. Apply rehearsal technique to balance, ensemble coordination, and pacing with a collaborator. 3. Communicate interpretive decisions clearly to collaborating musicians. 4. Perform prepared repertoire with a collaborative pianist in juries and recitals.</t>
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Prepare repertoire with a collaborative pianist, marking and rehearsing entrances, cutoffs, tempo, and balance.
+2. Apply articulation, phrasing, and intonation decisions to the delivery of the repertoire.
+3. Rehearse and perform with a collaborative pianist, responding to the accompaniment in the moment.
+4. Document the preparation of a work from first rehearsal to performance.</t>
           </r>
         </is>
       </c>
@@ -4977,17 +5019,71 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add: Units may not be used towards the Music Major or Minor.</t>
+            <t xml:space="preserve">classification records a 1-2 unit range where each unit carries the classification
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to MUS 281 and carries no level marker
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+learning outcomes are identical to MUS 281, MUS 282, and MUS 482, are written for applied study, and name the primary instrument on a vocal course
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+repeat cap differs across the coaching series
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -5008,7 +5104,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>Individual coaching with a faculty coach on repertoire requiring a collaborative pianist, for students enrolled in upper division applied study. Coaching times are arranged according to degree recital expectations. Requirements appear in the Music Student Handbook.</t>
+            <t>Individual vocal coaching with a collaborative pianist for music majors and minors at the upper division performance level, in preparation for the junior and senior recitals. Coaching times arranged according to the expectations in the Music Student Handbook.</t>
           </r>
           <r>
             <rPr>
@@ -5016,17 +5112,20 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Prepare repertoire with a collaborative pianist to a performance standard. 2. Apply rehearsal technique to balance, ensemble coordination, and pacing with a collaborator. 3. Communicate interpretive decisions clearly to collaborating musicians. 4. Perform prepared repertoire with a collaborative pianist in juries and recitals.</t>
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Build a recital program with a collaborative pianist, taking responsibility for repertoire, order, and pacing.
+2. Apply diction, translation, and poetic interpretation across repertoire in more than one language.
+3. Lead rehearsals with a collaborative pianist, setting the interpretive decisions and revising them across the preparation.
+4. Perform a program that meets the recital requirements in the Music Student Handbook.</t>
           </r>
         </is>
       </c>
@@ -5116,17 +5215,71 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no credit restriction published, though the handbook states coaching units do not count toward graduation requirements
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add: Units may not be used towards the Music Major or Minor.</t>
+            <t xml:space="preserve">classification records a 1-2 unit range where each unit carries the classification
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to MUS 282 and carries no level marker
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+learning outcomes are identical to MUS 281, MUS 282, and MUS 481 and are written for applied study
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+repeat cap differs across the coaching series
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -5147,7 +5300,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>Individual coaching with a faculty coach on repertoire requiring a collaborative pianist, for students enrolled in upper division applied study. Coaching times are arranged according to degree recital expectations. Requirements appear in the Music Student Handbook.</t>
+            <t>Individual instrumental coaching with a collaborative pianist for music majors and minors at the upper division performance level, in preparation for the junior and senior recitals. Coaching times arranged according to the expectations in the Music Student Handbook.</t>
           </r>
           <r>
             <rPr>
@@ -5155,17 +5308,20 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-outcomes are the generic applied study set, and outcome 2 addresses tone production on the primary instrument
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. Prepare repertoire with a collaborative pianist to a performance standard. 2. Apply rehearsal technique to balance, ensemble coordination, and pacing with a collaborator. 3. Communicate interpretive decisions clearly to collaborating musicians. 4. Perform prepared repertoire with a collaborative pianist in juries and recitals.</t>
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Build a recital program with a collaborative pianist, taking responsibility for repertoire, order, and pacing.
+2. Apply articulation, phrasing, intonation, and stylistic decisions across repertoire from more than one period.
+3. Lead rehearsals with a collaborative pianist, setting the interpretive decisions and revising them across the preparation.
+4. Perform a program that meets the recital requirements in the Music Student Handbook.</t>
           </r>
         </is>
       </c>
@@ -5472,17 +5628,17 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1-3 where the record holds 1
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1-3</t>
+            <t xml:space="preserve">record holds 1 unit where the catalog publishes 1–3
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>correct the record to 1–3</t>
           </r>
           <r>
             <rPr>
@@ -5490,21 +5646,98 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-record holds 1 unit where the catalog and handbook give 1–3
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>correct the record to 1–3</t>
-          </r>
-        </is>
-      </c>
-      <c r="T46" s="4" t="n"/>
+credit restriction keeps internship units off the major and minor
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the credit restriction</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is the university-wide internship text, shared with every department
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+learning outcomes state that outcomes vary
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+        </is>
+      </c>
+      <c r="T46" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Supervised work in a music-related organization or with a working musician, arranged through the department. Students hold assigned responsibilities and report on the placement.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Apply musical, technical, and organizational skills from the curriculum in a working setting.
+2. Hold assigned responsibilities and meet the deadlines the placement sets.
+3. Communicate with supervisors, colleagues, and audiences in the conventions of the workplace.
+4. Document the work completed and what it contributed to the organization.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6348,9 +6581,65 @@
             </rPr>
             <t>remove or apply it across the series</t>
           </r>
-        </is>
-      </c>
-      <c r="T57" s="4" t="n"/>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to MUS 660B and does not name voice
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+repeat cap differs across the coaching series
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
+          </r>
+        </is>
+      </c>
+      <c r="T57" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Individual vocal coaching with a collaborative pianist for graduate students, in preparation for the graduate recital. Coaching times arranged according to the expectations in the Graduate Student Handbook.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="58" ht="140" customHeight="1" s="12">
       <c r="A58" s="4" t="inlineStr">
@@ -6462,9 +6751,65 @@
             </rPr>
             <t>remove or apply it across the series</t>
           </r>
-        </is>
-      </c>
-      <c r="T58" s="4" t="n"/>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is identical to MUS 660A and does not name instruments
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+repeat cap differs across the coaching series
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
+          </r>
+        </is>
+      </c>
+      <c r="T58" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Individual instrumental coaching with a collaborative pianist for graduate students, in preparation for the graduate recital. Coaching times arranged according to the expectations in the Graduate Student Handbook.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="59" ht="140" customHeight="1" s="12">
       <c r="A59" s="6" t="inlineStr">
@@ -7049,7 +7394,7 @@
       <c r="T65" s="6" t="n"/>
     </row>
     <row r="66" s="12">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>MUS 698</t>
         </is>
@@ -7059,60 +7404,157 @@
           <t>Internship</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>Music: Graduate Studies</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr">
         <is>
           <t>1–3</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>blank</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>Formal advanced work opportunities integrating the academic program with their career aspirations. Integral advanced hands-on experience enhancing education and preparing for professional and personal success.</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>Department consent and minimum 2.0 GPA.</t>
         </is>
       </c>
-      <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="n"/>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="H66" s="4" t="n"/>
+      <c r="I66" s="4" t="n"/>
+      <c r="J66" s="4" t="inlineStr">
         <is>
           <t>May be repeated with department consent for a maximum of 6 units.</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K66" s="4" t="inlineStr">
         <is>
           <t>CR/NC grading only.</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="L66" s="4" t="inlineStr">
         <is>
           <t>On-ground.</t>
         </is>
       </c>
-      <c r="M66" s="2" t="n"/>
-      <c r="N66" s="2" t="inlineStr">
+      <c r="M66" s="4" t="n"/>
+      <c r="N66" s="4" t="inlineStr">
         <is>
           <t>No units may be applied to the Music major; no more than 3 units may be applied to the Music</t>
         </is>
       </c>
-      <c r="O66" s="2" t="n"/>
-      <c r="P66" s="2" t="n"/>
-      <c r="Q66" s="2" t="n"/>
-      <c r="R66" s="2" t="n"/>
-      <c r="S66" s="3" t="n"/>
-      <c r="T66" s="3" t="n"/>
+      <c r="O66" s="4" t="n"/>
+      <c r="P66" s="4" t="n"/>
+      <c r="Q66" s="4" t="n"/>
+      <c r="R66" s="4" t="n"/>
+      <c r="S66" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">no proposal on record in the Curriculog archive under 698 or a predecessor number
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>confirm with APS where the record sits</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description is the university-wide internship text with advanced inserted twice
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no learning outcomes published
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add learning outcomes</t>
+          </r>
+        </is>
+      </c>
+      <c r="T66" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Supervised professional work in a music-related organization, arranged through the department. Students hold assigned responsibilities at a level consistent with graduate study and report on the placement.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Apply graduate-level musical and professional skills in a working setting.
+2. Hold assigned responsibilities and meet the deadlines the placement sets.
+3. Communicate with supervisors, colleagues, and audiences in the conventions of the workplace.
+4. Evaluate the placement against the aims of the degree and their own professional plans.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="67" ht="112" customHeight="1" s="12">
       <c r="A67" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Correct the coaching classification form and repeat caps
The classification records the published unit range: C36 1-2u. MUS 481 and
482 already hold it and their finding is dropped. MUS 281 and 282 move from
S36 1u, and MUS 660A and 660B from C36 1u.

The repeat caps stand as published: 4 units at the lower division, 8 at the
upper division and the graduate level. The findings that changed them are
removed.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3047,7 +3047,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>reclassify to C36 1u</t>
+            <t>reclassify to C36 1-2u</t>
           </r>
           <r>
             <rPr>
@@ -3084,24 +3084,6 @@
               <sz val="10"/>
             </rPr>
             <t>revise the learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeat cap differs across the coaching series
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -3261,7 +3243,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>reclassify to C36 1u</t>
+            <t>reclassify to C36 1-2u</t>
           </r>
           <r>
             <rPr>
@@ -3298,24 +3280,6 @@
               <sz val="10"/>
             </rPr>
             <t>revise the learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeat cap differs across the coaching series
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -5019,25 +4983,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">classification records a 1-2 unit range where each unit carries the classification
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set the classification to C36 1u</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-description is identical to MUS 281 and carries no level marker
+            <t xml:space="preserve">description is identical to MUS 281 and carries no level marker
 </t>
           </r>
           <r>
@@ -5066,24 +5012,6 @@
               <sz val="10"/>
             </rPr>
             <t>revise the learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeat cap differs across the coaching series
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -5215,25 +5143,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">classification records a 1-2 unit range where each unit carries the classification
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set the classification to C36 1u</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-description is identical to MUS 282 and carries no level marker
+            <t xml:space="preserve">description is identical to MUS 282 and carries no level marker
 </t>
           </r>
           <r>
@@ -5262,24 +5172,6 @@
               <sz val="10"/>
             </rPr>
             <t>revise the learning outcomes</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeat cap differs across the coaching series
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -6569,7 +6461,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent, absent on most graduate applied courses
 </t>
           </r>
           <r>
@@ -6598,24 +6508,6 @@
               <sz val="10"/>
             </rPr>
             <t>revise the description</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeat cap differs across the coaching series
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>
@@ -6721,7 +6613,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">requires MUS 669, renumbered or discontinued
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+requires MUS 669, renumbered or discontinued
 </t>
           </r>
           <r>
@@ -6768,24 +6678,6 @@
               <sz val="10"/>
             </rPr>
             <t>revise the description</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-repeat cap differs across the coaching series
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set repeatability to may be repeated for credit for a maximum of 16 units</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Release the row heights on the course inventory sheet
Forty-one rows carried a fixed height with the custom-height flag set and
no longer sized to their content. The heights are cleared and the rows fit
their text again. The header row keeps its 30-point height.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -6473,7 +6473,7 @@
       <c r="T9" s="3"/>
       <c r="U9" s="2"/>
     </row>
-    <row r="10" spans="2:21" ht="126" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
         <v>79</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="2:21" ht="224" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B11" s="4" t="s">
         <v>88</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="12" spans="2:21" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
         <v>97</v>
       </c>
@@ -6627,7 +6627,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="2:21" ht="238" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
         <v>104</v>
       </c>
@@ -6679,7 +6679,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="2:21" ht="196" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
         <v>110</v>
       </c>
@@ -6727,7 +6727,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="2:21" ht="252" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
         <v>117</v>
       </c>
@@ -6873,7 +6873,7 @@
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
     </row>
-    <row r="18" spans="1:21" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B18" s="4" t="s">
         <v>141</v>
       </c>
@@ -6927,7 +6927,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="210" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B19" s="4" t="s">
         <v>151</v>
       </c>
@@ -6979,7 +6979,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="252" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B20" s="4" t="s">
         <v>158</v>
       </c>
@@ -7075,7 +7075,7 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
     </row>
-    <row r="22" spans="1:21" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
         <v>169</v>
       </c>
@@ -7129,7 +7129,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B23" s="4" t="s">
         <v>181</v>
       </c>
@@ -7391,7 +7391,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
     </row>
-    <row r="28" spans="1:21" ht="266" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B28" s="4" t="s">
         <v>214</v>
       </c>
@@ -7491,7 +7491,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="30" spans="1:21" s="12" customFormat="1" ht="126" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:21" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
         <v>797</v>
       </c>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="U30" s="6"/>
     </row>
-    <row r="31" spans="1:21" s="12" customFormat="1" ht="126" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:21" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="17" t="s">
         <v>797</v>
       </c>
@@ -7633,7 +7633,7 @@
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
     </row>
-    <row r="33" spans="1:21" s="11" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="17"/>
       <c r="B33" s="4" t="s">
         <v>249</v>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="U33" s="4"/>
     </row>
-    <row r="34" spans="1:21" ht="70" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B34" s="4" t="s">
         <v>256</v>
       </c>
@@ -7730,7 +7730,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="35" spans="1:21" s="12" customFormat="1" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="17" t="s">
         <v>797</v>
       </c>
@@ -7825,7 +7825,7 @@
       <c r="T36" s="3"/>
       <c r="U36" s="2"/>
     </row>
-    <row r="37" spans="1:21" ht="293" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B37" s="4" t="s">
         <v>276</v>
       </c>
@@ -7917,7 +7917,7 @@
       <c r="T38" s="2"/>
       <c r="U38" s="2"/>
     </row>
-    <row r="39" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B39" s="2" t="s">
         <v>287</v>
       </c>
@@ -8007,7 +8007,7 @@
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
     </row>
-    <row r="41" spans="1:21" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B41" s="4" t="s">
         <v>296</v>
       </c>
@@ -8061,7 +8061,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B42" s="4" t="s">
         <v>303</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B43" s="2" t="s">
         <v>306</v>
       </c>
@@ -8161,7 +8161,7 @@
       <c r="T43" s="2"/>
       <c r="U43" s="2"/>
     </row>
-    <row r="44" spans="1:21" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B44" s="2" t="s">
         <v>312</v>
       </c>
@@ -8255,7 +8255,7 @@
       <c r="T45" s="3"/>
       <c r="U45" s="3"/>
     </row>
-    <row r="46" spans="1:21" s="11" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="17"/>
       <c r="B46" s="4" t="s">
         <v>324</v>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="U47" s="2"/>
     </row>
-    <row r="48" spans="1:21" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B48" s="2" t="s">
         <v>343</v>
       </c>
@@ -8402,7 +8402,7 @@
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
     </row>
-    <row r="49" spans="1:21" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B49" s="2" t="s">
         <v>350</v>
       </c>
@@ -8446,7 +8446,7 @@
       <c r="T49" s="2"/>
       <c r="U49" s="2"/>
     </row>
-    <row r="50" spans="1:21" ht="145" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B50" s="4" t="s">
         <v>354</v>
       </c>
@@ -8490,7 +8490,7 @@
       <c r="T50" s="4"/>
       <c r="U50" s="4"/>
     </row>
-    <row r="51" spans="1:21" ht="148" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B51" s="4" t="s">
         <v>357</v>
       </c>
@@ -8578,7 +8578,7 @@
       <c r="T52" s="2"/>
       <c r="U52" s="2"/>
     </row>
-    <row r="53" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B53" s="2" t="s">
         <v>365</v>
       </c>
@@ -8622,7 +8622,7 @@
       <c r="T53" s="2"/>
       <c r="U53" s="2"/>
     </row>
-    <row r="54" spans="1:21" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B54" s="2" t="s">
         <v>370</v>
       </c>
@@ -8760,7 +8760,7 @@
       <c r="T56" s="2"/>
       <c r="U56" s="2"/>
     </row>
-    <row r="57" spans="1:21" ht="146" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B57" s="4" t="s">
         <v>387</v>
       </c>
@@ -8812,7 +8812,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="166" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B58" s="4" t="s">
         <v>395</v>
       </c>
@@ -8864,7 +8864,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="59" spans="1:21" s="20" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:21" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="16"/>
       <c r="B59" s="18" t="s">
         <v>402</v>
@@ -8913,7 +8913,7 @@
       <c r="T59" s="19"/>
       <c r="U59" s="18"/>
     </row>
-    <row r="60" spans="1:21" s="20" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:21" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="16"/>
       <c r="B60" s="18" t="s">
         <v>410</v>
@@ -8960,7 +8960,7 @@
       <c r="T60" s="19"/>
       <c r="U60" s="19"/>
     </row>
-    <row r="61" spans="1:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B61" s="2" t="s">
         <v>414</v>
       </c>
@@ -9004,7 +9004,7 @@
       <c r="T61" s="3"/>
       <c r="U61" s="3"/>
     </row>
-    <row r="62" spans="1:21" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A62" s="17" t="s">
         <v>797</v>
       </c>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="U62" s="9"/>
     </row>
-    <row r="63" spans="1:21" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A63" s="17" t="s">
         <v>797</v>
       </c>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="U63" s="8"/>
     </row>
-    <row r="64" spans="1:21" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B64" s="4" t="s">
         <v>433</v>
       </c>
@@ -9154,7 +9154,7 @@
       </c>
       <c r="U64" s="4"/>
     </row>
-    <row r="65" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B65" s="6" t="s">
         <v>440</v>
       </c>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="U65" s="6"/>
     </row>
-    <row r="66" spans="1:21" ht="167" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B66" s="4" t="s">
         <v>445</v>
       </c>
@@ -9250,7 +9250,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="67" spans="1:21" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A67" s="17" t="s">
         <v>797</v>
       </c>

</xml_diff>